<commit_message>
update two new student
</commit_message>
<xml_diff>
--- a/Data/評分表_總表.xlsx
+++ b/Data/評分表_總表.xlsx
@@ -26,12 +26,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="連浡崴_平靜" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="邵靖榕_快樂" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="鍾佩蓉_恐懼" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳子怡_平靜" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳怡瑾_平靜" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳翰博_悲傷" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="顏士傑_憤怒" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黃政文_恐懼" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黃鈺倢_渴望" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳奕廷_快樂" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳子怡_平靜" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳怡瑾_平靜" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳翰博_悲傷" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="陳陽安_恐懼" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="顏士傑_憤怒" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黃政文_恐懼" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黃鈺倢_渴望" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3557,7 +3559,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>陳子怡_平靜</t>
+          <t>陳奕廷_快樂</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -3578,7 +3580,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>得分 (4.8★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -3610,12 +3612,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>首輪即附參考照片並明確給出主題「泡沫之境」、平靜感受、滑鼠互動與自適應，意圖與載體對應清楚；後續逐輪追加日期變色、聲音、點擊變色與質感、三圖對應三風格，拆解有層次。</t>
+          <t>首輪即把「快樂」拆成五點抽象靈感與五點實際描述（輕飄飄／扭動／驚喜磁吸／天馬行空彈跳／多巴胺色彩），並明確給出 PANTONE 色號、液態玻璃、背景漸層、滑鼠拖移與線條行為；第二輪「感覺跟理想中效果差距蠻大的，我們一步一步做修改」並列五點具體項（背景亮藍、拿掉高斯模糊改 iOS 液態、白點像蝴蝶、線條五公分與頻率三分之一、三線中心吸成圓），意圖與技術需求一致。</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>「請參考照片的效果幫我生成出網頁，帶給人們平靜的感受」「主題名稱：泡沫之境 | The Land of Foam」「要能用滑鼠去與畫面互動。網頁大小要自適應」</t>
+          <t>「你現在是互動網頁的設計師，要把我給的靈感做成一個.html網頁並提供程式碼」「基本條件 1.網頁大小要自適應 2.做成.html網頁 3.讓人心情感到快樂的網站」「輕飄飄的感覺、扭動身體、會突然發現驚喜、天馬行空的創意、眼睛看出去的顏色是多巴胺」「用氣球被風吹過的感覺」「線條會像磁吸一樣，碰到就吸在一起，最多用三條線組合成球」「要液態玻璃的感覺」「點擊滑鼠左鍵在螢幕拖移會出現高斯模糊的波浪線條」；「感覺跟理想中效果差距蠻大的，我們一步一步做修改」「1.背景顏色換上亮藍色，晴朗天氣的天空 2.高斯模糊拿掉，液態玻璃效果指的是 iOS 26.3 圖標的液態效果 3.背後放模糊的白色小點點隨機飄動像蝴蝶 4.線條要像五公分長、出現頻率三分之一 5.三條線的中心吸在一起朝三角度，外圍連在一起會變成圓形」</t>
         </is>
       </c>
     </row>
@@ -3637,12 +3639,12 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>從參考圖與「泡沫之境」延伸出高斯模糊、噪點紋理、極簡排版與藍色彌散光感；後續以三張範例圖鎖定琥珀／霓虹／黑白三種質感與配色，視覺轉譯到位，情緒內涵一致。</t>
+          <t>從「快樂、多巴胺、輕飄飄、磁吸驚喜、液態玻璃」轉譯為 Canvas 波浪線、PANTONE 色、亮藍漸層、白點飄動、三線中心交疊與隨機反彈；第二輪後改為 iOS 風玻璃透亮、線條長度與頻率收斂；後續彩蛋碰碰樂、消除模式、輕快抖動與風力變速，情緒內涵與視覺一致。</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>「琥珀的質感、配色換成圖1範例，霓虹的質感、配色換成圖2範例，黑白的質感、配色換成圖3範例」；AI 復刻「高斯模糊、噪點紋理、彌散光感」</t>
+          <t>「液態玻璃」「多巴胺、充滿活力」「輕飄飄」「磁吸、三條線組合成球」「大波浪、小波浪、快速波浪」；AI 實作 globalCompositeOperation、filter、PANTONE 色、背景 Dots、LiquidLine 扭動與 group 磁吸、eggMode 碰碰樂、邊界反彈與數量上限</t>
         </is>
       </c>
     </row>
@@ -3659,17 +3661,17 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>每輪需求多能具體描述（日期變色＋聲音、點擊變色＋質感＋音效、三圖對應）；音效部分曾多輪來回（合成音→免費音效→連結失效→改本地檔），但能簡潔指出「太難聽」「沒有出現音樂」「點擊無法進去」並提供自找音樂檔名，最終收斂。</t>
+          <t>首輪即得完整 HTML 與設計對應；第二輪一句「一步一步做修改」搭配五點編號，每點皆可執行；後續「沒講到的就不要動，顏色、畫面呈現很讚」、觸控、消除模式、線條長度與抖動頻率等，指令簡潔、迭代有節奏。</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>「請幫我把旁邊的文字內容、色彩，可以隨著每天不同的日期而改變，並在這個基礎上加入聲音」；「生成出的音效太難聽了…請生成出能夠帶給人平靜、祥和的感受的音樂」；「沒有出現音樂，請仔細確認」</t>
+          <t>「感覺跟理想中效果差距蠻大的，我們一步一步做修改」+ 五點；「4.沒講到的就不要動，顏色、畫面呈現很讚」；多輪針對中心交接、風力、彩蛋、觸控、消除、輕快感逐一修正</t>
         </is>
       </c>
     </row>
@@ -3691,12 +3693,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>首輪即要求自適應；後續涉及音訊解鎖、CORS／連結失效時能與 AI 協作改為本地音檔與簡化載入邏輯，對瀏覽器與使用情境有考量。</t>
+          <t>需求含自適應、滑鼠拖移、觸控；實作具 resize、mousedown/touchstart/touchmove、邊界 margin、particles 數量上限 150、彩蛋觸發條件與組合球碰撞，環境與互動完整。</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>「網頁大小要自適應」；「出現新的問題，目前點擊無法進去，請直接刪掉目前html上音效的部分，以下是我找的音樂：（檔名）」；AI 處理 autoplay、CORS、本地檔</t>
+          <t>「網頁大小要自適應，跟著不同使用者的視窗大小進行調整」「點擊滑鼠左鍵在螢幕拖移」；AI 實作 resize()、handleInput、touch 事件、updatePhysics 邊界、particles.length &gt; 150、isEliminationMode</t>
         </is>
       </c>
     </row>
@@ -3718,19 +3720,19 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>能吸收並沿用「高斯模糊」「噪點紋理」「質感」「配色」等語彙，並以「圖1／圖2／圖3範例」精準對應三種風格；後續與 AI 討論音效時觸及 CORS、連結穩定性與本地檔，語彙內化清楚。</t>
+          <t>能運用「自適應」「PANTONE」「液態玻璃」「磁吸」「驚喜球」「高斯模糊」「多巴胺」；並接受「iOS 圖標液態效果」「輕飄飄」「像蝴蝶」「三條線中心交疊、外圍連成圓形」等描述，後續使用「抖動」「輕快」「彩蛋」等語彙，生字內化與演化清楚。</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>「琥珀的質感、配色換成圖1範例…」；「聲音一樣太難聽了，請直接搜索免費音效來搭配，最好可以跟大自然做連結」</t>
+          <t>「PANTONE 115c、orange 021c、volor 0621c（幫我修正）、Red0331c、green 0921c」「液態玻璃的感覺」「輕飄飄、扭動、磁吸、天馬行空」；「液態玻璃效果指的是 iOS 26.3 中圖標的液態效果」；AI 回「彩蛋觸發」「變速隨機風感」「輕快感」</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>陳怡瑾_平靜</t>
+          <t>陳子怡_平靜</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -3751,7 +3753,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>得分 (5.0★)</t>
+          <t>得分 (4.8★)</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3783,12 +3785,12 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>首輪即明確給出三項規範：自適應網頁、滑鼠左鍵點擊產生水波紋、滑鼠移動時水波隨風飄逸；後續逐步追加不用圖片改程式運算、點擊要明顯光亮、點點構成水波、附圖底色、日式青綠、花瓣累積與飄動、光隨點擊、同色系光暈與櫻花淺色，意圖拆解有層次。</t>
+          <t>首輪即附參考照片並明確給出主題「泡沫之境」、平靜感受、滑鼠互動與自適應，意圖與載體對應清楚；後續逐輪追加日期變色、聲音、點擊變色與質感、三圖對應三風格，拆解有層次。</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>「我想要作互動式網頁，要符合以下規範：自適應網頁、用滑鼠左鍵點擊產生水波紋、用滑鼠移動水波紋隨風飄逸的感覺」；「可以不要用圖片改用程式碼運算嗎？」</t>
+          <t>「請參考照片的效果幫我生成出網頁，帶給人們平靜的感受」「主題名稱：泡沫之境 | The Land of Foam」「要能用滑鼠去與畫面互動。網頁大小要自適應」</t>
         </is>
       </c>
     </row>
@@ -3810,12 +3812,12 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>從「平靜」水波延伸出程序化水藍漸層、點點粒子水波、明顯光亮、附圖底色、日式青綠／抹茶色、落花堆積與隨風飄動、點擊時光暈與水波同步、同色系光暈、櫻花兩色淺而有差異，視覺與情緒轉譯到位。</t>
+          <t>從參考圖與「泡沫之境」延伸出高斯模糊、噪點紋理、極簡排版與藍色彌散光感；後續以三張範例圖鎖定琥珀／霓虹／黑白三種質感與配色，視覺轉譯到位，情緒內涵一致。</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>「我希望滑鼠點擊時水波可以特別一點 (有明顯光亮)」；「背景顏色可以偏青綠色嗎？想要有點小日式的感覺」；「光的感覺我希望隨水波滑鼠點擊產生」；「點擊的光暈可以改成同色系嗎？」</t>
+          <t>「琥珀的質感、配色換成圖1範例，霓虹的質感、配色換成圖2範例，黑白的質感、配色換成圖3範例」；AI 復刻「高斯模糊、噪點紋理、彌散光感」</t>
         </is>
       </c>
     </row>
@@ -3832,17 +3834,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>多輪指令皆具體且一次鎖定一兩個改動：沒畫面→接受 AI 說明改網路圖/程式運算；明顯光亮、點點構成水波、附圖底色、青綠日式與花瓣累積、花瓣隨風、光隨點擊、同色系、櫻花深一點再微調兩色淺一點，迭代節奏清楚。</t>
+          <t>每輪需求多能具體描述（日期變色＋聲音、點擊變色＋質感＋音效、三圖對應）；音效部分曾多輪來回（合成音→免費音效→連結失效→改本地檔），但能簡潔指出「太難聽」「沒有出現音樂」「點擊無法進去」並提供自找音樂檔名，最終收斂。</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>「網頁沒有畫面」；「我的點點是想要構成水波而不是背景」；「有幾個想要修正：背景顏色可以偏青綠色嗎？想要有點小日式的感覺、掉落的花瓣可以累積在螢幕下面嗎？」；「累積的花瓣希望也可以隨風飄動」</t>
+          <t>「請幫我把旁邊的文字內容、色彩，可以隨著每天不同的日期而改變，並在這個基礎上加入聲音」；「生成出的音效太難聽了…請生成出能夠帶給人平靜、祥和的感受的音樂」；「沒有出現音樂，請仔細確認」</t>
         </is>
       </c>
     </row>
@@ -3864,12 +3866,12 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>首輪即要求自適應；遇到 WebGL 本地檔案限制導致沒畫面時，能接受 AI 說明並改用網路圖片測試或改為純程式運算，對瀏覽器限制與除錯情境有配合。</t>
+          <t>首輪即要求自適應；後續涉及音訊解鎖、CORS／連結失效時能與 AI 協作改為本地音檔與簡化載入邏輯，對瀏覽器與使用情境有考量。</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>「自適應網頁」；「網頁沒有畫面」→ AI 說明 file:/// 與 WebGL 限制、提供 Live Server／Base64／網路圖測試；「可以不要用圖片改用程式碼運算嗎？」徹底避開讀檔問題</t>
+          <t>「網頁大小要自適應」；「出現新的問題，目前點擊無法進去，請直接刪掉目前html上音效的部分，以下是我找的音樂：（檔名）」；AI 處理 autoplay、CORS、本地檔</t>
         </is>
       </c>
     </row>
@@ -3891,19 +3893,19 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>能吸收並沿用「自適應」「程式碼運算」「光暈」「同色系」「程序化」等語彙，並以「點點構成水波」「隨風飄逸」「明顯光亮」「日式感覺」等描述與 AI 對齊視覺，內化與演化清楚。</t>
+          <t>能吸收並沿用「高斯模糊」「噪點紋理」「質感」「配色」等語彙，並以「圖1／圖2／圖3範例」精準對應三種風格；後續與 AI 討論音效時觸及 CORS、連結穩定性與本地檔，語彙內化清楚。</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>「可以不要用圖片改用程式碼運算嗎？」；「點擊的光暈可以改成同色系嗎？」；「櫻花的顏色兩個可以再淺一點嗎？兩者顏色有一點差異」；AI 回覆中的「程序化生成」「物理堆積系統」等詞在後續對話中對應</t>
+          <t>「琥珀的質感、配色換成圖1範例…」；「聲音一樣太難聽了，請直接搜索免費音效來搭配，最好可以跟大自然做連結」</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>陳翰博_悲傷</t>
+          <t>陳怡瑾_平靜</t>
         </is>
       </c>
       <c r="B161" t="inlineStr"/>
@@ -3924,7 +3926,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>得分 (4.6★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -3956,12 +3958,12 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>將「散去後的悲傷」轉譯為粒子擴散、煙霧淡化、滑鼠痕跡與 Perlin Noise，並主動請求具象化物體靈感（蒲公英殘骸、餘燼、墨痕等），意圖與隱喻對應精準。</t>
+          <t>首輪即明確給出三項規範：自適應網頁、滑鼠左鍵點擊產生水波紋、滑鼠移動時水波隨風飄逸；後續逐步追加不用圖片改程式運算、點擊要明顯光亮、點點構成水波、附圖底色、日式青綠、花瓣累積與飄動、光隨點擊、同色系光暈與櫻花淺色，意圖拆解有層次。</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔（內含必要的css 和javascript），另外關於&lt;散去後的悲傷&gt;你有什麼具象化的物體名稱也提供給我靈感」</t>
+          <t>「我想要作互動式網頁，要符合以下規範：自適應網頁、用滑鼠左鍵點擊產生水波紋、用滑鼠移動水波紋隨風飄逸的感覺」；「可以不要用圖片改用程式碼運算嗎？」</t>
         </is>
       </c>
     </row>
@@ -3983,12 +3985,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>結合 p5.js 粒子、半透明覆蓋與聽覺設計（41.2Hz 三角波、Sub Bass、正弦波合成器），「記憶如煙花散去」與低頻震盪的氛圍一致；具象化名單直接啟發情感層次。</t>
+          <t>從「平靜」水波延伸出程序化水藍漸層、點點粒子水波、明顯光亮、附圖底色、日式青綠／抹茶色、落花堆積與隨風飄動、點擊時光暈與水波同步、同色系光暈、櫻花兩色淺而有差異，視覺與情緒轉譯到位。</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>「接下來疊加音樂效果我希望添加像是 sub bass 或 sine wave與合成器音色，來立體化氛圍空間-在滑鼠靠近時隨著形狀浮現並散去」</t>
+          <t>「我希望滑鼠點擊時水波可以特別一點 (有明顯光亮)」；「背景顏色可以偏青綠色嗎？想要有點小日式的感覺」；「光的感覺我希望隨水波滑鼠點擊產生」；「點擊的光暈可以改成同色系嗎？」</t>
         </is>
       </c>
     </row>
@@ -4005,17 +4007,17 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>以「散去後的悲傷」單一主題開場並索求靈感與程式碼，AI 一次給出粒子系統與具象化名單；追加音訊時明確描述「滑鼠靠近時隨著形狀浮現並散去」，迭代方向清楚。</t>
+          <t>多輪指令皆具體且一次鎖定一兩個改動：沒畫面→接受 AI 說明改網路圖/程式運算；明顯光亮、點點構成水波、附圖底色、青綠日式與花瓣累積、花瓣隨風、光隨點擊、同色系、櫻花深一點再微調兩色淺一點，迭代節奏清楚。</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔」；「疊加音樂效果…sub bass 或 sine wave與合成器音色」</t>
+          <t>「網頁沒有畫面」；「我的點點是想要構成水波而不是背景」；「有幾個想要修正：背景顏色可以偏青綠色嗎？想要有點小日式的感覺、掉落的花瓣可以累積在螢幕下面嗎？」；「累積的花瓣希望也可以隨風飄動」</t>
         </is>
       </c>
     </row>
@@ -4032,17 +4034,17 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>需求含網頁互動、即時創作轉 HTML、自適應與音訊觸發（使用者點擊後啟動）；程式中有 start-screen、點擊閾值與 Golden 粒子等設計，環境與互動考量完整。</t>
+          <t>首輪即要求自適應；遇到 WebGL 本地檔案限制導致沒畫面時，能接受 AI 說明並改用網路圖片測試或改為純程式運算，對瀏覽器限制與除錯情境有配合。</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>提供 openprocessing 及時創作檔案並要求轉 HTML；音訊設計含「使用者點擊後才能啟動」的引導畫面</t>
+          <t>「自適應網頁」；「網頁沒有畫面」→ AI 說明 file:/// 與 WebGL 限制、提供 Live Server／Base64／網路圖測試；「可以不要用圖片改用程式碼運算嗎？」徹底避開讀檔問題</t>
         </is>
       </c>
     </row>
@@ -4064,19 +4066,19 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>能吸收並反饋「Perlin Noise」「Sub Bass」「Triangle 波形」「BiquadFilter」「exponentialRampToValueAtTime」等術語，並以「41.2Hz 三角波震盪，記憶如煙花散去」整合聽覺與視覺敘事。</t>
+          <t>能吸收並沿用「自適應」「程式碼運算」「光暈」「同色系」「程序化」等語彙，並以「點點構成水波」「隨風飄逸」「明顯光亮」「日式感覺」等描述與 AI 對齊視覺，內化與演化清楚。</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>對話中接納「粒子系統」「低頻深沉音」「動態過濾」等描述並進一步要求疊加音樂效果</t>
+          <t>「可以不要用圖片改用程式碼運算嗎？」；「點擊的光暈可以改成同色系嗎？」；「櫻花的顏色兩個可以再淺一點嗎？兩者顏色有一點差異」；AI 回覆中的「程序化生成」「物理堆積系統」等詞在後續對話中對應</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>顏士傑_憤怒</t>
+          <t>陳翰博_悲傷</t>
         </is>
       </c>
       <c r="B169" t="inlineStr"/>
@@ -4097,7 +4099,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>得分 (4.8★)</t>
+          <t>得分 (4.6★)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4119,7 +4121,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4129,12 +4131,12 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>首輪即用五維（顏色、形狀、質感、明暗、空間）拆解憤怒：深紅、鋸齒齒輪、粗糙／黑板／毛氈、暗沉無光、狹隘；具體意象為心臟在中央被齒輪包圍摩擦、左鍵點擊齒輪轉動、簡單2D、HTML 含 CSS/JS，並主動請 AI 提供憤怒具象化物體靈感，意圖與視覺邏輯一致。</t>
+          <t>將「散去後的悲傷」轉譯為粒子擴散、煙霧淡化、滑鼠痕跡與 Perlin Noise，並主動請求具象化物體靈感（蒲公英殘骸、餘燼、墨痕等），意圖與隱喻對應精準。</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>「我選的情緒是憤怒」「用顏色,形狀,質感,明暗,空間來表達憤怒，顏色是深紅色,形狀是鋸齒齒輪,質感是粗糙,像黑板的材質,毛氈，明暗是有點暗沉無光，空間是狹隘」「有顆暗沉無光且深紅的心臟在網頁的正中央，被四周帶有多齒的鋸齒齒輪包圍且摩擦著」「滑鼠左鍵在鋸齒圖上點擊，所有鋸齒都會一起轉動，設計成簡單2Ｄ即可，給我HTML檔（內含必要的css 和javascript），另外關於憤怒你有什麼具象化的物體名稱也提供給我靈感」</t>
+          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔（內含必要的css 和javascript），另外關於&lt;散去後的悲傷&gt;你有什麼具象化的物體名稱也提供給我靈感」</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4148,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4156,12 +4158,12 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>從深紅心臟、鋸齒齒輪、粗糙毛氈、狹隘空間轉譯為漸層與粗糙線條、齒輪毛髮線條、岩漿／血液粒子、心臟跳動與點擊加速、齒輪減速摩擦；主動引用 AI brainstorm 依序加入放射狀裂痕、心臟火環、鐵籠邊框，內部爆發與外在囚禁的對比強，審美與憤怒的壓迫／爆發感對應佳。</t>
+          <t>結合 p5.js 粒子、半透明覆蓋與聽覺設計（41.2Hz 三角波、Sub Bass、正弦波合成器），「記憶如煙花散去」與低頻震盪的氛圍一致；具象化名單直接啟發情感層次。</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>「深紅色」「鋸齒齒輪」「粗糙」「毛氈」「暗沉無光」「狹隘」「心臟的四周會偶爾出現橘紅色的岩漿」「心臟都會變大又變小」「點擊時…鮮紅色的particle」「齒輪…變慢（增加摩擦心臟的感覺）」；「缺少了一些你上面brain storm的idea, 比如說lava, burning, cage」→ 先做1（裂痕）、接著做2（火環）、做3（鐵籠）</t>
+          <t>「接下來疊加音樂效果我希望添加像是 sub bass 或 sine wave與合成器音色，來立體化氛圍空間-在滑鼠靠近時隨著形狀浮現並散去」</t>
         </is>
       </c>
     </row>
@@ -4173,22 +4175,22 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>首輪一次給足五維與互動、技術需求；第二輪補響應式、心臟畫大、距離小、岩漿；第三輪心臟位置、跳動、點擊加速、鮮紅粒子、齒輪變慢；第四輪心臟 Y 軸置中；第五輪主動問「怎麼安排 graphic」後依序要求裂痕、火環、鐵籠；遇 script error 明確說「重來」並獲乾淨版本；最後一輪微調齒輪轉速對比。迭代有節奏、需求具體。</t>
+          <t>以「散去後的悲傷」單一主題開場並索求靈感與程式碼，AI 一次給出粒子系統與具象化名單；追加音訊時明確描述「滑鼠靠近時隨著形狀浮現並散去」，迭代方向清楚。</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>「響應式設計」「心臟畫大一點」「齒輪之間距離很小，幾乎有摩擦的感覺」「橘紅色的岩漿」；「心臟放在四個齒輪的正中間」「心臟變大又變小」「mouse left button click時…心臟…頻率暫時加速」「齒輪…變慢」；「重來，你遇到script error了」；「在還沒有按下mouse 之前，讓齒輪轉得比現在快一點」</t>
+          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔」；「疊加音樂效果…sub bass 或 sine wave與合成器音色」</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4202,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4210,12 +4212,12 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>需求含響應式、左鍵互動、多裝置／觸控；實作具 resize、心臟跳動與點擊加速、齒輪減速、岩漿／血液粒子、放射狀裂痕、火環、鐵籠、轉速對比，視覺層次與互動完整；技術面為逐步追加而非一次預見，故略扣一星。</t>
+          <t>需求含網頁互動、即時創作轉 HTML、自適應與音訊觸發（使用者點擊後啟動）；程式中有 start-screen、點擊閾值與 Golden 粒子等設計，環境與互動考量完整。</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>「可以在任何的device打開都不失format」；AI 實作響應式、觸控、心臟跳動邏輯、齒輪減速、裂痕／火環／鐵籠繪製、轉速參數調整</t>
+          <t>提供 openprocessing 及時創作檔案並要求轉 HTML；音訊設計含「使用者點擊後才能啟動」的引導畫面</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4229,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4237,19 +4239,19 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>能運用「質感」「明暗」「空間」「狹隘」「毛氈」「岩漿」「響應式」「心臟跳動」「齒輪摩擦」等語彙，並接受「壓抑的爆發」「摩擦壓迫感」等描述；主動引用 AI 提供的 brainstorm（lava, burning, cage）要求依序實作，生字內化與視覺演化清楚。</t>
+          <t>能吸收並反饋「Perlin Noise」「Sub Bass」「Triangle 波形」「BiquadFilter」「exponentialRampToValueAtTime」等術語，並以「41.2Hz 三角波震盪，記憶如煙花散去」整合聽覺與視覺敘事。</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>「質感是粗糙,像黑板的材質,毛氈」「空間是狹隘」「岩漿」；「缺少了一些你上面brain storm的idea, 比如說lava, burning file, cage」→ 先做1、接著做2、做3</t>
+          <t>對話中接納「粒子系統」「低頻深沉音」「動態過濾」等描述並進一步要求疊加音樂效果</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>黃政文_恐懼</t>
+          <t>陳陽安_恐懼</t>
         </is>
       </c>
       <c r="B177" t="inlineStr"/>
@@ -4270,7 +4272,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>得分 (4.2★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -4292,7 +4294,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4302,12 +4304,12 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>將「恐懼」具象化為呼吸式縮放、裂痕、長按層級、暗角與有機輪廓，規範完整且具互動藝術與氛圍感；需求條列清晰，技術方案（Canvas、CSS Variables、狀態管理）對應明確。</t>
+          <t>首輪即以「專業藝術互動式網頁設計師」身份給出完整場景：轉輪水龍頭、玻璃杯接水、水位上升、杯子破碎、拱火燃燒、水澆滅火焰，以及「按住關閉、鬆開開啟」的互動邏輯；後續能拆解圖層與視覺順序（「所有物品和動畫必須使用兩層以上圖層」「波浪圖層必須在洪水圖層上、高度必須高於洪水、去掉 ripple、泡泡最高高度和洪水同高」），意圖與技術對應明確。</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>「我想要作互動式網頁，要符合以下規範：他是自適應網頁…滑鼠移動 &gt; 背景產生局部扭曲…長按 10 秒 &gt; 輪廓透明 25%…滾動 100% &gt; 畫面出現中央選擇區塊」</t>
+          <t>「我需要你以非常專業的藝術互動式網頁設計師的身份幫我製作一個 html 網站」「最左邊轉輪式水龍頭、出水口正下方透明玻璃杯、水龍頭開啟時出水口有水的動畫流到杯子裡、杯子裡的水用動畫讓水位上升、達到最高水平面後杯子破碎、杯子下方拱火燃燒、杯子破碎後液體澆滅火焰」「轉輪開關默認開啟，除非一直按住才逐漸關閉，鬆開鼠標左鍵又逐漸開啟」；「所有物品和動畫必須使用兩層以上的圖層去製作，每個圖層的顏色深度必須不一樣」「波浪圖層必須在洪水圖層上，並且高度必須高於洪水，必須看得見波浪的動畫效果，去掉 ripple，泡泡的最高高度也和洪水同一個高度」</t>
         </is>
       </c>
     </row>
@@ -4319,22 +4321,22 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>以「氛圍感」「Atmospheric Horror」定位視覺風格，要求無裂痕/無輪廓的初始態與漸進揭露；後續接受程序化生成取代圖片，具象化有機輪廓與扭曲效果。</t>
+          <t>從「恐懼／壓迫」轉譯為雨、水龍頭、玻璃杯、水位上升、破碎、火焰熄滅、洪水淹沒、多層波浪與泡泡；學生要求「兩層以上圖層、顏色深度不一、火焰更真實、雨水不穿透杯底」，AI 實作多層雨、雙層玻璃杯、三層火焰、雙層洪水波浪、水霧與泡泡，情緒與視覺流程一致。</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+          <t>「轉輪式水龍頭」「透明玻璃杯」「水流動畫」「杯子破碎動畫」「拱火燃燒、搖曳」「水澆滅火焰」；「兩層以上圖層、顏色深度必須不一樣」「火焰再更真實一些」；AI 實作 rainLayer 三層、glassBack/glassFront、多層火焰與波浪、flood 與 surface 分層</t>
         </is>
       </c>
     </row>
@@ -4346,22 +4348,22 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>一次給足完整規範，AI 回覆即提供結構化方案與程式碼；追加「不用圖片、程式碼運算」與「完整 HTML」時能快速收斂為單一檔案實作。</t>
+          <t>首輪即給足場景與互動邏輯，獲得完整 HTML；後續每輪指令具體可執行（「兩層以上圖層…全部加下去」「波浪圖層必須在洪水圖層上…去掉 ripple…泡泡最高高度和洪水同高」），迭代有節奏、不發散。</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+          <t>「所有物品和動畫必須使用兩層以上的圖層去製作…並且將就剛剛的建議全部加下去」；「波浪圖層必須在洪水圖層上，並且高度必須高於洪水，必須看得見波浪的動畫效果，去掉 ripple，泡泡的最高高度也和洪水同一個高度，我這裡指的波浪圖層是那個多個深淺顏色不一的圖層製造的波浪效果」</t>
         </is>
       </c>
     </row>
@@ -4373,22 +4375,22 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>需求已含自適應、多種輸入（滑鼠移動/點擊/長按/滾輪）與狀態累積（裂痕永久、輪廓殘留）；AI 建議震動動畫、效能最佳化與遮罩圖使用，具產品思維。</t>
+          <t>需求含視窗自適應、圖層順序與高度同步、雨水不穿透杯底；對話中明確要求「水不會繼續往下流」「進入杯子裡的雨水都不會到達杯子的底部以下」「波浪圖層在洪水圖層上、高度高於洪水」「泡泡最高高度和洪水同高」，環境與技術預見完整。</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>規範中已明確「自適應網頁」「滑鼠左鍵點擊（單擊）」「長按 1 秒 &gt; 畫面微震動」等層級與恢復條件</t>
+          <t>「默認開啟、除非一直按住才逐漸關閉」；「被杯子接住的水不會繼續往下流，所有進入杯子裡的雨水都不會到達杯子的底部以下」；「波浪圖層必須在洪水圖層上」「泡泡的最高高度也和洪水同一個高度」；AI 實作完全窗口自適應、flood/surface 結構、bubble 生成限制</t>
         </is>
       </c>
     </row>
@@ -4400,29 +4402,29 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>能運用「程序化生成」「Backdrop-filter」「Simplex Noise」等術語與 AI 回覆中的技術建議；需求從圖片改為純程式運算時表述清楚。</t>
+          <t>能運用「藝術互動式網頁設計師」「圖層」「顏色深度」「洪水」「波浪」「ripple」「動畫」等語彙，並精準描述圖層順序與高度關係（「波浪圖層必須在洪水圖層上」「高度必須高於洪水」「泡泡最高高度和洪水同高」），吸收 AI 回覆中的結構說明後再提出修正，生字內化與演化清楚。</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」；對話中接受「Vanilla JS 搭配 CSS Variables」「requestAnimationFrame」等用語</t>
+          <t>「專業的藝術互動式網頁設計師」「轉輪式水龍頭」「水位上升」「杯子破碎」「拱火」「澆滅」；「兩層以上的圖層」「每個圖層的顏色深度必須不一樣」；「波浪圖層必須在洪水圖層上」「多個深淺顏色不一的圖層製造的波浪效果」「去掉 ripple」</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>黃鈺倢_渴望</t>
+          <t>顏士傑_憤怒</t>
         </is>
       </c>
       <c r="B185" t="inlineStr"/>
@@ -4443,7 +4445,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>得分 (5.0★)</t>
+          <t>得分 (4.8★)</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -4465,7 +4467,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4475,12 +4477,12 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>首輪給出互動響應式網頁；後續多次附參考圖並具體描述：實體地勢圖、前進感（光點變大）、時間變色明顯、多層山河依手繪線各自高度與流動、色彩繽紛可調 ramp，意圖與技術載體對應清楚。</t>
+          <t>首輪即用五維（顏色、形狀、質感、明暗、空間）拆解憤怒：深紅、鋸齒齒輪、粗糙／黑板／毛氈、暗沉無光、狹隘；具體意象為心臟在中央被齒輪包圍摩擦、左鍵點擊齒輪轉動、簡單2D、HTML 含 CSS/JS，並主動請 AI 提供憤怒具象化物體靈感，意圖與視覺邏輯一致。</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>「我要做一個互動響應式html網頁」；「第一層的山河要像這樣有實體的地勢圖…要有真的在前進的感覺，所以光點要離自己越來越近(大)」「背景要隨著時間改變顏色這點請做得明顯一點」</t>
+          <t>「我選的情緒是憤怒」「用顏色,形狀,質感,明暗,空間來表達憤怒，顏色是深紅色,形狀是鋸齒齒輪,質感是粗糙,像黑板的材質,毛氈，明暗是有點暗沉無光，空間是狹隘」「有顆暗沉無光且深紅的心臟在網頁的正中央，被四周帶有多齒的鋸齒齒輪包圍且摩擦著」「滑鼠左鍵在鋸齒圖上點擊，所有鋸齒都會一起轉動，設計成簡單2Ｄ即可，給我HTML檔（內含必要的css 和javascript），另外關於憤怒你有什麼具象化的物體名稱也提供給我靈感」</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4494,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -4502,12 +4504,12 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>從參考圖與「渴望」行進感延伸出實體地勢、多層山河帶、各自 ramp 繽紛色、通道不透明與羽化、天空漸層日夜變色、黑夜飽和度 0 灰階、自訂日夜色盤與前進 Zoom In，視覺與情緒轉譯到位。</t>
+          <t>從深紅心臟、鋸齒齒輪、粗糙毛氈、狹隘空間轉譯為漸層與粗糙線條、齒輪毛髮線條、岩漿／血液粒子、心臟跳動與點擊加速、齒輪減速摩擦；主動引用 AI brainstorm 依序加入放射狀裂痕、心臟火環、鐵籠邊框，內部爆發與外在囚禁的對比強，審美與憤怒的壓迫／爆發感對應佳。</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>「請類似照我用不同顏色畫的線做成各有不同高度起伏的山河，並且要有自然流動感…色彩各自繽紛(而且我能自己調整顏色ramp)」；「我想要天空是漸層的…日夜變色…黑夜時整個畫面飽和度0」</t>
+          <t>「深紅色」「鋸齒齒輪」「粗糙」「毛氈」「暗沉無光」「狹隘」「心臟的四周會偶爾出現橘紅色的岩漿」「心臟都會變大又變小」「點擊時…鮮紅色的particle」「齒輪…變慢（增加摩擦心臟的感覺）」；「缺少了一些你上面brain storm的idea, 比如說lava, burning, cage」→ 先做1（裂痕）、接著做2（火環）、做3（鐵籠）</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4521,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4529,12 +4531,12 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>多輪指令多能具體鎖定要改項目：明顯一點、拿掉 UI 改後台調、夜日改成慢慢變回日、通道不透明跟羽化、加 saturation、前進感 Zoom In；偶有「幫我改」但多附圖或前後文，迭代節奏清楚。</t>
+          <t>首輪一次給足五維與互動、技術需求；第二輪補響應式、心臟畫大、距離小、岩漿；第三輪心臟位置、跳動、點擊加速、鮮紅粒子、齒輪變慢；第四輪心臟 Y 軸置中；第五輪主動問「怎麼安排 graphic」後依序要求裂痕、火環、鐵籠；遇 script error 明確說「重來」並獲乾淨版本；最後一輪微調齒輪轉速對比。迭代有節奏、需求具體。</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>「夜日更替的瞬間太硬了(黑夜直接瞬間變白)，請改成慢慢變回日」；「還有我想要讓他是不透明的，跟羽化的」；「好 記得幫我加上saturation值」；「我想要改成整體有前進的感覺(Zoom In)」</t>
+          <t>「響應式設計」「心臟畫大一點」「齒輪之間距離很小，幾乎有摩擦的感覺」「橘紅色的岩漿」；「心臟放在四個齒輪的正中間」「心臟變大又變小」「mouse left button click時…心臟…頻率暫時加速」「齒輪…變慢」；「重來，你遇到script error了」；「在還沒有按下mouse 之前，讓齒輪轉得比現在快一點」</t>
         </is>
       </c>
     </row>
@@ -4546,22 +4548,22 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>首輪即要求響應式；後續主動要求「可調整的 UI 拿掉、自己在後台調就好」，並在天空/日夜/通道等處皆採後台參數，對作品呈現與除錯情境有預見。</t>
+          <t>需求含響應式、左鍵互動、多裝置／觸控；實作具 resize、心臟跳動與點擊加速、齒輪減速、岩漿／血液粒子、放射狀裂痕、火環、鐵籠、轉速對比，視覺層次與互動完整；技術面為逐步追加而非一次預見，故略扣一星。</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>「網頁大小要自適應」；「我不想要讓那個可以調整的UI直接出現在網頁上 拿掉好了 我自己在後台調就好」；AI 以 STATE/global 後台參數對應</t>
+          <t>「可以在任何的device打開都不失format」；AI 實作響應式、觸控、心臟跳動邏輯、齒輪減速、裂痕／火環／鐵籠繪製、轉速參數調整</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4575,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4583,10 +4585,356 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
+          <t>能運用「質感」「明暗」「空間」「狹隘」「毛氈」「岩漿」「響應式」「心臟跳動」「齒輪摩擦」等語彙，並接受「壓抑的爆發」「摩擦壓迫感」等描述；主動引用 AI 提供的 brainstorm（lava, burning, cage）要求依序實作，生字內化與視覺演化清楚。</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>「質感是粗糙,像黑板的材質,毛氈」「空間是狹隘」「岩漿」；「缺少了一些你上面brain storm的idea, 比如說lava, burning file, cage」→ 先做1、接著做2、做3</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>黃政文_恐懼</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr"/>
+      <c r="C193" t="inlineStr"/>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>評分項目</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>使用 AI</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>得分 (4.2★)</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>犀利點評</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>原文擷取 (學生指令)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>意圖解析與拆解</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>將「恐懼」具象化為呼吸式縮放、裂痕、長按層級、暗角與有機輪廓，規範完整且具互動藝術與氛圍感；需求條列清晰，技術方案（Canvas、CSS Variables、狀態管理）對應明確。</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>「我想要作互動式網頁，要符合以下規範：他是自適應網頁…滑鼠移動 &gt; 背景產生局部扭曲…長按 10 秒 &gt; 輪廓透明 25%…滾動 100% &gt; 畫面出現中央選擇區塊」</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>審美轉譯與內涵</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>以「氛圍感」「Atmospheric Horror」定位視覺風格，要求無裂痕/無輪廓的初始態與漸進揭露；後續接受程序化生成取代圖片，具象化有機輪廓與扭曲效果。</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>溝通效率與迭代</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>一次給足完整規範，AI 回覆即提供結構化方案與程式碼；追加「不用圖片、程式碼運算」與「完整 HTML」時能快速收斂為單一檔案實作。</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>環境預見與判斷</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>需求已含自適應、多種輸入（滑鼠移動/點擊/長按/滾輪）與狀態累積（裂痕永久、輪廓殘留）；AI 建議震動動畫、效能最佳化與遮罩圖使用，具產品思維。</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>規範中已明確「自適應網頁」「滑鼠左鍵點擊（單擊）」「長按 1 秒 &gt; 畫面微震動」等層級與恢復條件</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>生字內化與演化</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>能運用「程序化生成」「Backdrop-filter」「Simplex Noise」等術語與 AI 回覆中的技術建議；需求從圖片改為純程式運算時表述清楚。</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」；對話中接受「Vanilla JS 搭配 CSS Variables」「requestAnimationFrame」等用語</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>黃鈺倢_渴望</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr"/>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>評分項目</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>使用 AI</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>得分 (5.0★)</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>犀利點評</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>原文擷取 (學生指令)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>意圖解析與拆解</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>首輪給出互動響應式網頁；後續多次附參考圖並具體描述：實體地勢圖、前進感（光點變大）、時間變色明顯、多層山河依手繪線各自高度與流動、色彩繽紛可調 ramp，意圖與技術載體對應清楚。</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>「我要做一個互動響應式html網頁」；「第一層的山河要像這樣有實體的地勢圖…要有真的在前進的感覺，所以光點要離自己越來越近(大)」「背景要隨著時間改變顏色這點請做得明顯一點」</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>審美轉譯與內涵</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>從參考圖與「渴望」行進感延伸出實體地勢、多層山河帶、各自 ramp 繽紛色、通道不透明與羽化、天空漸層日夜變色、黑夜飽和度 0 灰階、自訂日夜色盤與前進 Zoom In，視覺與情緒轉譯到位。</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>「請類似照我用不同顏色畫的線做成各有不同高度起伏的山河，並且要有自然流動感…色彩各自繽紛(而且我能自己調整顏色ramp)」；「我想要天空是漸層的…日夜變色…黑夜時整個畫面飽和度0」</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>溝通效率與迭代</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>多輪指令多能具體鎖定要改項目：明顯一點、拿掉 UI 改後台調、夜日改成慢慢變回日、通道不透明跟羽化、加 saturation、前進感 Zoom In；偶有「幫我改」但多附圖或前後文，迭代節奏清楚。</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>「夜日更替的瞬間太硬了(黑夜直接瞬間變白)，請改成慢慢變回日」；「還有我想要讓他是不透明的，跟羽化的」；「好 記得幫我加上saturation值」；「我想要改成整體有前進的感覺(Zoom In)」</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>環境預見與判斷</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>首輪即要求響應式；後續主動要求「可調整的 UI 拿掉、自己在後台調就好」，並在天空/日夜/通道等處皆採後台參數，對作品呈現與除錯情境有預見。</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>「網頁大小要自適應」；「我不想要讓那個可以調整的UI直接出現在網頁上 拿掉好了 我自己在後台調就好」；AI 以 STATE/global 後台參數對應</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>生字內化與演化</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
           <t>能運用並吸收「顏色 ramp」「stops」「飽和度」「日夜變色」「漸層」「羽化」「dayPhase」「saturation」等語彙，並以「後台調整」「多層山河」「各有高度起伏」精準描述需求，內化與演化清楚。</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
+      <c r="E207" t="inlineStr">
         <is>
           <t>「色彩各自繽紛(而且我能自己調整顏色ramp)」；「希望在黑夜時可以整個畫面顏色直接也變成飽和度0那樣」；「我可以自己選擇日夜顏色慢慢變化時會有哪些顏色嗎？」</t>
         </is>
@@ -6555,7 +6903,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>得分 (4.8★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -6587,12 +6935,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>首輪即附參考照片並明確給出主題「泡沫之境」、平靜感受、滑鼠互動與自適應，意圖與載體對應清楚；後續逐輪追加日期變色、聲音、點擊變色與質感、三圖對應三風格，拆解有層次。</t>
+          <t>首輪即把「快樂」拆成五點抽象靈感與五點實際描述（輕飄飄／扭動／驚喜磁吸／天馬行空彈跳／多巴胺色彩），並明確給出 PANTONE 色號、液態玻璃、背景漸層、滑鼠拖移與線條行為；第二輪「感覺跟理想中效果差距蠻大的，我們一步一步做修改」並列五點具體項（背景亮藍、拿掉高斯模糊改 iOS 液態、白點像蝴蝶、線條五公分與頻率三分之一、三線中心吸成圓），意圖與技術需求一致。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>「請參考照片的效果幫我生成出網頁，帶給人們平靜的感受」「主題名稱：泡沫之境 | The Land of Foam」「要能用滑鼠去與畫面互動。網頁大小要自適應」</t>
+          <t>「你現在是互動網頁的設計師，要把我給的靈感做成一個.html網頁並提供程式碼」「基本條件 1.網頁大小要自適應 2.做成.html網頁 3.讓人心情感到快樂的網站」「輕飄飄的感覺、扭動身體、會突然發現驚喜、天馬行空的創意、眼睛看出去的顏色是多巴胺」「用氣球被風吹過的感覺」「線條會像磁吸一樣，碰到就吸在一起，最多用三條線組合成球」「要液態玻璃的感覺」「點擊滑鼠左鍵在螢幕拖移會出現高斯模糊的波浪線條」；「感覺跟理想中效果差距蠻大的，我們一步一步做修改」「1.背景顏色換上亮藍色，晴朗天氣的天空 2.高斯模糊拿掉，液態玻璃效果指的是 iOS 26.3 圖標的液態效果 3.背後放模糊的白色小點點隨機飄動像蝴蝶 4.線條要像五公分長、出現頻率三分之一 5.三條線的中心吸在一起朝三角度，外圍連在一起會變成圓形」</t>
         </is>
       </c>
     </row>
@@ -6614,12 +6962,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>從參考圖與「泡沫之境」延伸出高斯模糊、噪點紋理、極簡排版與藍色彌散光感；後續以三張範例圖鎖定琥珀／霓虹／黑白三種質感與配色，視覺轉譯到位，情緒內涵一致。</t>
+          <t>從「快樂、多巴胺、輕飄飄、磁吸驚喜、液態玻璃」轉譯為 Canvas 波浪線、PANTONE 色、亮藍漸層、白點飄動、三線中心交疊與隨機反彈；第二輪後改為 iOS 風玻璃透亮、線條長度與頻率收斂；後續彩蛋碰碰樂、消除模式、輕快抖動與風力變速，情緒內涵與視覺一致。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>「琥珀的質感、配色換成圖1範例，霓虹的質感、配色換成圖2範例，黑白的質感、配色換成圖3範例」；AI 復刻「高斯模糊、噪點紋理、彌散光感」</t>
+          <t>「液態玻璃」「多巴胺、充滿活力」「輕飄飄」「磁吸、三條線組合成球」「大波浪、小波浪、快速波浪」；AI 實作 globalCompositeOperation、filter、PANTONE 色、背景 Dots、LiquidLine 扭動與 group 磁吸、eggMode 碰碰樂、邊界反彈與數量上限</t>
         </is>
       </c>
     </row>
@@ -6636,17 +6984,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>每輪需求多能具體描述（日期變色＋聲音、點擊變色＋質感＋音效、三圖對應）；音效部分曾多輪來回（合成音→免費音效→連結失效→改本地檔），但能簡潔指出「太難聽」「沒有出現音樂」「點擊無法進去」並提供自找音樂檔名，最終收斂。</t>
+          <t>首輪即得完整 HTML 與設計對應；第二輪一句「一步一步做修改」搭配五點編號，每點皆可執行；後續「沒講到的就不要動，顏色、畫面呈現很讚」、觸控、消除模式、線條長度與抖動頻率等，指令簡潔、迭代有節奏。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>「請幫我把旁邊的文字內容、色彩，可以隨著每天不同的日期而改變，並在這個基礎上加入聲音」；「生成出的音效太難聽了…請生成出能夠帶給人平靜、祥和的感受的音樂」；「沒有出現音樂，請仔細確認」</t>
+          <t>「感覺跟理想中效果差距蠻大的，我們一步一步做修改」+ 五點；「4.沒講到的就不要動，顏色、畫面呈現很讚」；多輪針對中心交接、風力、彩蛋、觸控、消除、輕快感逐一修正</t>
         </is>
       </c>
     </row>
@@ -6668,12 +7016,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>首輪即要求自適應；後續涉及音訊解鎖、CORS／連結失效時能與 AI 協作改為本地音檔與簡化載入邏輯，對瀏覽器與使用情境有考量。</t>
+          <t>需求含自適應、滑鼠拖移、觸控；實作具 resize、mousedown/touchstart/touchmove、邊界 margin、particles 數量上限 150、彩蛋觸發條件與組合球碰撞，環境與互動完整。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>「網頁大小要自適應」；「出現新的問題，目前點擊無法進去，請直接刪掉目前html上音效的部分，以下是我找的音樂：（檔名）」；AI 處理 autoplay、CORS、本地檔</t>
+          <t>「網頁大小要自適應，跟著不同使用者的視窗大小進行調整」「點擊滑鼠左鍵在螢幕拖移」；AI 實作 resize()、handleInput、touch 事件、updatePhysics 邊界、particles.length &gt; 150、isEliminationMode</t>
         </is>
       </c>
     </row>
@@ -6695,12 +7043,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>能吸收並沿用「高斯模糊」「噪點紋理」「質感」「配色」等語彙，並以「圖1／圖2／圖3範例」精準對應三種風格；後續與 AI 討論音效時觸及 CORS、連結穩定性與本地檔，語彙內化清楚。</t>
+          <t>能運用「自適應」「PANTONE」「液態玻璃」「磁吸」「驚喜球」「高斯模糊」「多巴胺」；並接受「iOS 圖標液態效果」「輕飄飄」「像蝴蝶」「三條線中心交疊、外圍連成圓形」等描述，後續使用「抖動」「輕快」「彩蛋」等語彙，生字內化與演化清楚。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>「琥珀的質感、配色換成圖1範例…」；「聲音一樣太難聽了，請直接搜索免費音效來搭配，最好可以跟大自然做連結」</t>
+          <t>「PANTONE 115c、orange 021c、volor 0621c（幫我修正）、Red0331c、green 0921c」「液態玻璃的感覺」「輕飄飄、扭動、磁吸、天馬行空」；「液態玻璃效果指的是 iOS 26.3 中圖標的液態效果」；AI 回「彩蛋觸發」「變速隨機風感」「輕快感」</t>
         </is>
       </c>
     </row>
@@ -6731,7 +7079,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>得分 (5.0★)</t>
+          <t>得分 (4.8★)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -6763,12 +7111,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>首輪即明確給出三項規範：自適應網頁、滑鼠左鍵點擊產生水波紋、滑鼠移動時水波隨風飄逸；後續逐步追加不用圖片改程式運算、點擊要明顯光亮、點點構成水波、附圖底色、日式青綠、花瓣累積與飄動、光隨點擊、同色系光暈與櫻花淺色，意圖拆解有層次。</t>
+          <t>首輪即附參考照片並明確給出主題「泡沫之境」、平靜感受、滑鼠互動與自適應，意圖與載體對應清楚；後續逐輪追加日期變色、聲音、點擊變色與質感、三圖對應三風格，拆解有層次。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>「我想要作互動式網頁，要符合以下規範：自適應網頁、用滑鼠左鍵點擊產生水波紋、用滑鼠移動水波紋隨風飄逸的感覺」；「可以不要用圖片改用程式碼運算嗎？」</t>
+          <t>「請參考照片的效果幫我生成出網頁，帶給人們平靜的感受」「主題名稱：泡沫之境 | The Land of Foam」「要能用滑鼠去與畫面互動。網頁大小要自適應」</t>
         </is>
       </c>
     </row>
@@ -6790,12 +7138,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>從「平靜」水波延伸出程序化水藍漸層、點點粒子水波、明顯光亮、附圖底色、日式青綠／抹茶色、落花堆積與隨風飄動、點擊時光暈與水波同步、同色系光暈、櫻花兩色淺而有差異，視覺與情緒轉譯到位。</t>
+          <t>從參考圖與「泡沫之境」延伸出高斯模糊、噪點紋理、極簡排版與藍色彌散光感；後續以三張範例圖鎖定琥珀／霓虹／黑白三種質感與配色，視覺轉譯到位，情緒內涵一致。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>「我希望滑鼠點擊時水波可以特別一點 (有明顯光亮)」；「背景顏色可以偏青綠色嗎？想要有點小日式的感覺」；「光的感覺我希望隨水波滑鼠點擊產生」；「點擊的光暈可以改成同色系嗎？」</t>
+          <t>「琥珀的質感、配色換成圖1範例，霓虹的質感、配色換成圖2範例，黑白的質感、配色換成圖3範例」；AI 復刻「高斯模糊、噪點紋理、彌散光感」</t>
         </is>
       </c>
     </row>
@@ -6812,17 +7160,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>多輪指令皆具體且一次鎖定一兩個改動：沒畫面→接受 AI 說明改網路圖/程式運算；明顯光亮、點點構成水波、附圖底色、青綠日式與花瓣累積、花瓣隨風、光隨點擊、同色系、櫻花深一點再微調兩色淺一點，迭代節奏清楚。</t>
+          <t>每輪需求多能具體描述（日期變色＋聲音、點擊變色＋質感＋音效、三圖對應）；音效部分曾多輪來回（合成音→免費音效→連結失效→改本地檔），但能簡潔指出「太難聽」「沒有出現音樂」「點擊無法進去」並提供自找音樂檔名，最終收斂。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>「網頁沒有畫面」；「我的點點是想要構成水波而不是背景」；「有幾個想要修正：背景顏色可以偏青綠色嗎？想要有點小日式的感覺、掉落的花瓣可以累積在螢幕下面嗎？」；「累積的花瓣希望也可以隨風飄動」</t>
+          <t>「請幫我把旁邊的文字內容、色彩，可以隨著每天不同的日期而改變，並在這個基礎上加入聲音」；「生成出的音效太難聽了…請生成出能夠帶給人平靜、祥和的感受的音樂」；「沒有出現音樂，請仔細確認」</t>
         </is>
       </c>
     </row>
@@ -6844,12 +7192,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>首輪即要求自適應；遇到 WebGL 本地檔案限制導致沒畫面時，能接受 AI 說明並改用網路圖片測試或改為純程式運算，對瀏覽器限制與除錯情境有配合。</t>
+          <t>首輪即要求自適應；後續涉及音訊解鎖、CORS／連結失效時能與 AI 協作改為本地音檔與簡化載入邏輯，對瀏覽器與使用情境有考量。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>「自適應網頁」；「網頁沒有畫面」→ AI 說明 file:/// 與 WebGL 限制、提供 Live Server／Base64／網路圖測試；「可以不要用圖片改用程式碼運算嗎？」徹底避開讀檔問題</t>
+          <t>「網頁大小要自適應」；「出現新的問題，目前點擊無法進去，請直接刪掉目前html上音效的部分，以下是我找的音樂：（檔名）」；AI 處理 autoplay、CORS、本地檔</t>
         </is>
       </c>
     </row>
@@ -6871,12 +7219,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>能吸收並沿用「自適應」「程式碼運算」「光暈」「同色系」「程序化」等語彙，並以「點點構成水波」「隨風飄逸」「明顯光亮」「日式感覺」等描述與 AI 對齊視覺，內化與演化清楚。</t>
+          <t>能吸收並沿用「高斯模糊」「噪點紋理」「質感」「配色」等語彙，並以「圖1／圖2／圖3範例」精準對應三種風格；後續與 AI 討論音效時觸及 CORS、連結穩定性與本地檔，語彙內化清楚。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>「可以不要用圖片改用程式碼運算嗎？」；「點擊的光暈可以改成同色系嗎？」；「櫻花的顏色兩個可以再淺一點嗎？兩者顏色有一點差異」；AI 回覆中的「程序化生成」「物理堆積系統」等詞在後續對話中對應</t>
+          <t>「琥珀的質感、配色換成圖1範例…」；「聲音一樣太難聽了，請直接搜索免費音效來搭配，最好可以跟大自然做連結」</t>
         </is>
       </c>
     </row>
@@ -6907,7 +7255,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>得分 (4.6★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -6939,12 +7287,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>將「散去後的悲傷」轉譯為粒子擴散、煙霧淡化、滑鼠痕跡與 Perlin Noise，並主動請求具象化物體靈感（蒲公英殘骸、餘燼、墨痕等），意圖與隱喻對應精準。</t>
+          <t>首輪即明確給出三項規範：自適應網頁、滑鼠左鍵點擊產生水波紋、滑鼠移動時水波隨風飄逸；後續逐步追加不用圖片改程式運算、點擊要明顯光亮、點點構成水波、附圖底色、日式青綠、花瓣累積與飄動、光隨點擊、同色系光暈與櫻花淺色，意圖拆解有層次。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔（內含必要的css 和javascript），另外關於&lt;散去後的悲傷&gt;你有什麼具象化的物體名稱也提供給我靈感」</t>
+          <t>「我想要作互動式網頁，要符合以下規範：自適應網頁、用滑鼠左鍵點擊產生水波紋、用滑鼠移動水波紋隨風飄逸的感覺」；「可以不要用圖片改用程式碼運算嗎？」</t>
         </is>
       </c>
     </row>
@@ -6966,12 +7314,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>結合 p5.js 粒子、半透明覆蓋與聽覺設計（41.2Hz 三角波、Sub Bass、正弦波合成器），「記憶如煙花散去」與低頻震盪的氛圍一致；具象化名單直接啟發情感層次。</t>
+          <t>從「平靜」水波延伸出程序化水藍漸層、點點粒子水波、明顯光亮、附圖底色、日式青綠／抹茶色、落花堆積與隨風飄動、點擊時光暈與水波同步、同色系光暈、櫻花兩色淺而有差異，視覺與情緒轉譯到位。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>「接下來疊加音樂效果我希望添加像是 sub bass 或 sine wave與合成器音色，來立體化氛圍空間-在滑鼠靠近時隨著形狀浮現並散去」</t>
+          <t>「我希望滑鼠點擊時水波可以特別一點 (有明顯光亮)」；「背景顏色可以偏青綠色嗎？想要有點小日式的感覺」；「光的感覺我希望隨水波滑鼠點擊產生」；「點擊的光暈可以改成同色系嗎？」</t>
         </is>
       </c>
     </row>
@@ -6988,17 +7336,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>以「散去後的悲傷」單一主題開場並索求靈感與程式碼，AI 一次給出粒子系統與具象化名單；追加音訊時明確描述「滑鼠靠近時隨著形狀浮現並散去」，迭代方向清楚。</t>
+          <t>多輪指令皆具體且一次鎖定一兩個改動：沒畫面→接受 AI 說明改網路圖/程式運算；明顯光亮、點點構成水波、附圖底色、青綠日式與花瓣累積、花瓣隨風、光隨點擊、同色系、櫻花深一點再微調兩色淺一點，迭代節奏清楚。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔」；「疊加音樂效果…sub bass 或 sine wave與合成器音色」</t>
+          <t>「網頁沒有畫面」；「我的點點是想要構成水波而不是背景」；「有幾個想要修正：背景顏色可以偏青綠色嗎？想要有點小日式的感覺、掉落的花瓣可以累積在螢幕下面嗎？」；「累積的花瓣希望也可以隨風飄動」</t>
         </is>
       </c>
     </row>
@@ -7015,17 +7363,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>需求含網頁互動、即時創作轉 HTML、自適應與音訊觸發（使用者點擊後啟動）；程式中有 start-screen、點擊閾值與 Golden 粒子等設計，環境與互動考量完整。</t>
+          <t>首輪即要求自適應；遇到 WebGL 本地檔案限制導致沒畫面時，能接受 AI 說明並改用網路圖片測試或改為純程式運算，對瀏覽器限制與除錯情境有配合。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>提供 openprocessing 及時創作檔案並要求轉 HTML；音訊設計含「使用者點擊後才能啟動」的引導畫面</t>
+          <t>「自適應網頁」；「網頁沒有畫面」→ AI 說明 file:/// 與 WebGL 限制、提供 Live Server／Base64／網路圖測試；「可以不要用圖片改用程式碼運算嗎？」徹底避開讀檔問題</t>
         </is>
       </c>
     </row>
@@ -7047,12 +7395,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>能吸收並反饋「Perlin Noise」「Sub Bass」「Triangle 波形」「BiquadFilter」「exponentialRampToValueAtTime」等術語，並以「41.2Hz 三角波震盪，記憶如煙花散去」整合聽覺與視覺敘事。</t>
+          <t>能吸收並沿用「自適應」「程式碼運算」「光暈」「同色系」「程序化」等語彙，並以「點點構成水波」「隨風飄逸」「明顯光亮」「日式感覺」等描述與 AI 對齊視覺，內化與演化清楚。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>對話中接納「粒子系統」「低頻深沉音」「動態過濾」等描述並進一步要求疊加音樂效果</t>
+          <t>「可以不要用圖片改用程式碼運算嗎？」；「點擊的光暈可以改成同色系嗎？」；「櫻花的顏色兩個可以再淺一點嗎？兩者顏色有一點差異」；AI 回覆中的「程序化生成」「物理堆積系統」等詞在後續對話中對應</t>
         </is>
       </c>
     </row>
@@ -7083,7 +7431,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>得分 (4.8★)</t>
+          <t>得分 (4.6★)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -7105,7 +7453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7115,12 +7463,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>首輪即用五維（顏色、形狀、質感、明暗、空間）拆解憤怒：深紅、鋸齒齒輪、粗糙／黑板／毛氈、暗沉無光、狹隘；具體意象為心臟在中央被齒輪包圍摩擦、左鍵點擊齒輪轉動、簡單2D、HTML 含 CSS/JS，並主動請 AI 提供憤怒具象化物體靈感，意圖與視覺邏輯一致。</t>
+          <t>將「散去後的悲傷」轉譯為粒子擴散、煙霧淡化、滑鼠痕跡與 Perlin Noise，並主動請求具象化物體靈感（蒲公英殘骸、餘燼、墨痕等），意圖與隱喻對應精準。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>「我選的情緒是憤怒」「用顏色,形狀,質感,明暗,空間來表達憤怒，顏色是深紅色,形狀是鋸齒齒輪,質感是粗糙,像黑板的材質,毛氈，明暗是有點暗沉無光，空間是狹隘」「有顆暗沉無光且深紅的心臟在網頁的正中央，被四周帶有多齒的鋸齒齒輪包圍且摩擦著」「滑鼠左鍵在鋸齒圖上點擊，所有鋸齒都會一起轉動，設計成簡單2Ｄ即可，給我HTML檔（內含必要的css 和javascript），另外關於憤怒你有什麼具象化的物體名稱也提供給我靈感」</t>
+          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔（內含必要的css 和javascript），另外關於&lt;散去後的悲傷&gt;你有什麼具象化的物體名稱也提供給我靈感」</t>
         </is>
       </c>
     </row>
@@ -7132,7 +7480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7142,12 +7490,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>從深紅心臟、鋸齒齒輪、粗糙毛氈、狹隘空間轉譯為漸層與粗糙線條、齒輪毛髮線條、岩漿／血液粒子、心臟跳動與點擊加速、齒輪減速摩擦；主動引用 AI brainstorm 依序加入放射狀裂痕、心臟火環、鐵籠邊框，內部爆發與外在囚禁的對比強，審美與憤怒的壓迫／爆發感對應佳。</t>
+          <t>結合 p5.js 粒子、半透明覆蓋與聽覺設計（41.2Hz 三角波、Sub Bass、正弦波合成器），「記憶如煙花散去」與低頻震盪的氛圍一致；具象化名單直接啟發情感層次。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>「深紅色」「鋸齒齒輪」「粗糙」「毛氈」「暗沉無光」「狹隘」「心臟的四周會偶爾出現橘紅色的岩漿」「心臟都會變大又變小」「點擊時…鮮紅色的particle」「齒輪…變慢（增加摩擦心臟的感覺）」；「缺少了一些你上面brain storm的idea, 比如說lava, burning, cage」→ 先做1（裂痕）、接著做2（火環）、做3（鐵籠）</t>
+          <t>「接下來疊加音樂效果我希望添加像是 sub bass 或 sine wave與合成器音色，來立體化氛圍空間-在滑鼠靠近時隨著形狀浮現並散去」</t>
         </is>
       </c>
     </row>
@@ -7159,22 +7507,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>首輪一次給足五維與互動、技術需求；第二輪補響應式、心臟畫大、距離小、岩漿；第三輪心臟位置、跳動、點擊加速、鮮紅粒子、齒輪變慢；第四輪心臟 Y 軸置中；第五輪主動問「怎麼安排 graphic」後依序要求裂痕、火環、鐵籠；遇 script error 明確說「重來」並獲乾淨版本；最後一輪微調齒輪轉速對比。迭代有節奏、需求具體。</t>
+          <t>以「散去後的悲傷」單一主題開場並索求靈感與程式碼，AI 一次給出粒子系統與具象化名單；追加音訊時明確描述「滑鼠靠近時隨著形狀浮現並散去」，迭代方向清楚。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>「響應式設計」「心臟畫大一點」「齒輪之間距離很小，幾乎有摩擦的感覺」「橘紅色的岩漿」；「心臟放在四個齒輪的正中間」「心臟變大又變小」「mouse left button click時…心臟…頻率暫時加速」「齒輪…變慢」；「重來，你遇到script error了」；「在還沒有按下mouse 之前，讓齒輪轉得比現在快一點」</t>
+          <t>「我將創建一個網頁互動設計呈現&lt;散去後的悲傷&gt;…請轉給我HTML檔」；「疊加音樂效果…sub bass 或 sine wave與合成器音色」</t>
         </is>
       </c>
     </row>
@@ -7186,7 +7534,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -7196,12 +7544,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>需求含響應式、左鍵互動、多裝置／觸控；實作具 resize、心臟跳動與點擊加速、齒輪減速、岩漿／血液粒子、放射狀裂痕、火環、鐵籠、轉速對比，視覺層次與互動完整；技術面為逐步追加而非一次預見，故略扣一星。</t>
+          <t>需求含網頁互動、即時創作轉 HTML、自適應與音訊觸發（使用者點擊後啟動）；程式中有 start-screen、點擊閾值與 Golden 粒子等設計，環境與互動考量完整。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>「可以在任何的device打開都不失format」；AI 實作響應式、觸控、心臟跳動邏輯、齒輪減速、裂痕／火環／鐵籠繪製、轉速參數調整</t>
+          <t>提供 openprocessing 及時創作檔案並要求轉 HTML；音訊設計含「使用者點擊後才能啟動」的引導畫面</t>
         </is>
       </c>
     </row>
@@ -7213,7 +7561,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -7223,12 +7571,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>能運用「質感」「明暗」「空間」「狹隘」「毛氈」「岩漿」「響應式」「心臟跳動」「齒輪摩擦」等語彙，並接受「壓抑的爆發」「摩擦壓迫感」等描述；主動引用 AI 提供的 brainstorm（lava, burning, cage）要求依序實作，生字內化與視覺演化清楚。</t>
+          <t>能吸收並反饋「Perlin Noise」「Sub Bass」「Triangle 波形」「BiquadFilter」「exponentialRampToValueAtTime」等術語，並以「41.2Hz 三角波震盪，記憶如煙花散去」整合聽覺與視覺敘事。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>「質感是粗糙,像黑板的材質,毛氈」「空間是狹隘」「岩漿」；「缺少了一些你上面brain storm的idea, 比如說lava, burning file, cage」→ 先做1、接著做2、做3</t>
+          <t>對話中接納「粒子系統」「低頻深沉音」「動態過濾」等描述並進一步要求疊加音樂效果</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7607,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>得分 (4.2★)</t>
+          <t>得分 (5.0★)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -7281,7 +7629,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7291,12 +7639,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>將「恐懼」具象化為呼吸式縮放、裂痕、長按層級、暗角與有機輪廓，規範完整且具互動藝術與氛圍感；需求條列清晰，技術方案（Canvas、CSS Variables、狀態管理）對應明確。</t>
+          <t>首輪即以「專業藝術互動式網頁設計師」身份給出完整場景：轉輪水龍頭、玻璃杯接水、水位上升、杯子破碎、拱火燃燒、水澆滅火焰，以及「按住關閉、鬆開開啟」的互動邏輯；後續能拆解圖層與視覺順序（「所有物品和動畫必須使用兩層以上圖層」「波浪圖層必須在洪水圖層上、高度必須高於洪水、去掉 ripple、泡泡最高高度和洪水同高」），意圖與技術對應明確。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>「我想要作互動式網頁，要符合以下規範：他是自適應網頁…滑鼠移動 &gt; 背景產生局部扭曲…長按 10 秒 &gt; 輪廓透明 25%…滾動 100% &gt; 畫面出現中央選擇區塊」</t>
+          <t>「我需要你以非常專業的藝術互動式網頁設計師的身份幫我製作一個 html 網站」「最左邊轉輪式水龍頭、出水口正下方透明玻璃杯、水龍頭開啟時出水口有水的動畫流到杯子裡、杯子裡的水用動畫讓水位上升、達到最高水平面後杯子破碎、杯子下方拱火燃燒、杯子破碎後液體澆滅火焰」「轉輪開關默認開啟，除非一直按住才逐漸關閉，鬆開鼠標左鍵又逐漸開啟」；「所有物品和動畫必須使用兩層以上的圖層去製作，每個圖層的顏色深度必須不一樣」「波浪圖層必須在洪水圖層上，並且高度必須高於洪水，必須看得見波浪的動畫效果，去掉 ripple，泡泡的最高高度也和洪水同一個高度」</t>
         </is>
       </c>
     </row>
@@ -7308,22 +7656,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>以「氛圍感」「Atmospheric Horror」定位視覺風格，要求無裂痕/無輪廓的初始態與漸進揭露；後續接受程序化生成取代圖片，具象化有機輪廓與扭曲效果。</t>
+          <t>從「恐懼／壓迫」轉譯為雨、水龍頭、玻璃杯、水位上升、破碎、火焰熄滅、洪水淹沒、多層波浪與泡泡；學生要求「兩層以上圖層、顏色深度不一、火焰更真實、雨水不穿透杯底」，AI 實作多層雨、雙層玻璃杯、三層火焰、雙層洪水波浪、水霧與泡泡，情緒與視覺流程一致。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+          <t>「轉輪式水龍頭」「透明玻璃杯」「水流動畫」「杯子破碎動畫」「拱火燃燒、搖曳」「水澆滅火焰」；「兩層以上圖層、顏色深度必須不一樣」「火焰再更真實一些」；AI 實作 rainLayer 三層、glassBack/glassFront、多層火焰與波浪、flood 與 surface 分層</t>
         </is>
       </c>
     </row>
@@ -7335,22 +7683,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>一次給足完整規範，AI 回覆即提供結構化方案與程式碼；追加「不用圖片、程式碼運算」與「完整 HTML」時能快速收斂為單一檔案實作。</t>
+          <t>首輪即給足場景與互動邏輯，獲得完整 HTML；後續每輪指令具體可執行（「兩層以上圖層…全部加下去」「波浪圖層必須在洪水圖層上…去掉 ripple…泡泡最高高度和洪水同高」），迭代有節奏、不發散。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+          <t>「所有物品和動畫必須使用兩層以上的圖層去製作…並且將就剛剛的建議全部加下去」；「波浪圖層必須在洪水圖層上，並且高度必須高於洪水，必須看得見波浪的動畫效果，去掉 ripple，泡泡的最高高度也和洪水同一個高度，我這裡指的波浪圖層是那個多個深淺顏色不一的圖層製造的波浪效果」</t>
         </is>
       </c>
     </row>
@@ -7362,22 +7710,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>需求已含自適應、多種輸入（滑鼠移動/點擊/長按/滾輪）與狀態累積（裂痕永久、輪廓殘留）；AI 建議震動動畫、效能最佳化與遮罩圖使用，具產品思維。</t>
+          <t>需求含視窗自適應、圖層順序與高度同步、雨水不穿透杯底；對話中明確要求「水不會繼續往下流」「進入杯子裡的雨水都不會到達杯子的底部以下」「波浪圖層在洪水圖層上、高度高於洪水」「泡泡最高高度和洪水同高」，環境與技術預見完整。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>規範中已明確「自適應網頁」「滑鼠左鍵點擊（單擊）」「長按 1 秒 &gt; 畫面微震動」等層級與恢復條件</t>
+          <t>「默認開啟、除非一直按住才逐漸關閉」；「被杯子接住的水不會繼續往下流，所有進入杯子裡的雨水都不會到達杯子的底部以下」；「波浪圖層必須在洪水圖層上」「泡泡的最高高度也和洪水同一個高度」；AI 實作完全窗口自適應、flood/surface 結構、bubble 生成限制</t>
         </is>
       </c>
     </row>
@@ -7389,22 +7737,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>能運用「程序化生成」「Backdrop-filter」「Simplex Noise」等術語與 AI 回覆中的技術建議；需求從圖片改為純程式運算時表述清楚。</t>
+          <t>能運用「藝術互動式網頁設計師」「圖層」「顏色深度」「洪水」「波浪」「ripple」「動畫」等語彙，並精準描述圖層順序與高度關係（「波浪圖層必須在洪水圖層上」「高度必須高於洪水」「泡泡最高高度和洪水同高」），吸收 AI 回覆中的結構說明後再提出修正，生字內化與演化清楚。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>「不要用圖片改用程式碼運算」；對話中接受「Vanilla JS 搭配 CSS Variables」「requestAnimationFrame」等用語</t>
+          <t>「專業的藝術互動式網頁設計師」「轉輪式水龍頭」「水位上升」「杯子破碎」「拱火」「澆滅」；「兩層以上的圖層」「每個圖層的顏色深度必須不一樣」；「波浪圖層必須在洪水圖層上」「多個深淺顏色不一的圖層製造的波浪效果」「去掉 ripple」</t>
         </is>
       </c>
     </row>
@@ -7435,6 +7783,358 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>得分 (4.8★)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>犀利點評</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>原文擷取 (學生指令)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>意圖解析與拆解</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>首輪即用五維（顏色、形狀、質感、明暗、空間）拆解憤怒：深紅、鋸齒齒輪、粗糙／黑板／毛氈、暗沉無光、狹隘；具體意象為心臟在中央被齒輪包圍摩擦、左鍵點擊齒輪轉動、簡單2D、HTML 含 CSS/JS，並主動請 AI 提供憤怒具象化物體靈感，意圖與視覺邏輯一致。</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>「我選的情緒是憤怒」「用顏色,形狀,質感,明暗,空間來表達憤怒，顏色是深紅色,形狀是鋸齒齒輪,質感是粗糙,像黑板的材質,毛氈，明暗是有點暗沉無光，空間是狹隘」「有顆暗沉無光且深紅的心臟在網頁的正中央，被四周帶有多齒的鋸齒齒輪包圍且摩擦著」「滑鼠左鍵在鋸齒圖上點擊，所有鋸齒都會一起轉動，設計成簡單2Ｄ即可，給我HTML檔（內含必要的css 和javascript），另外關於憤怒你有什麼具象化的物體名稱也提供給我靈感」</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>審美轉譯與內涵</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>從深紅心臟、鋸齒齒輪、粗糙毛氈、狹隘空間轉譯為漸層與粗糙線條、齒輪毛髮線條、岩漿／血液粒子、心臟跳動與點擊加速、齒輪減速摩擦；主動引用 AI brainstorm 依序加入放射狀裂痕、心臟火環、鐵籠邊框，內部爆發與外在囚禁的對比強，審美與憤怒的壓迫／爆發感對應佳。</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>「深紅色」「鋸齒齒輪」「粗糙」「毛氈」「暗沉無光」「狹隘」「心臟的四周會偶爾出現橘紅色的岩漿」「心臟都會變大又變小」「點擊時…鮮紅色的particle」「齒輪…變慢（增加摩擦心臟的感覺）」；「缺少了一些你上面brain storm的idea, 比如說lava, burning, cage」→ 先做1（裂痕）、接著做2（火環）、做3（鐵籠）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>溝通效率與迭代</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>首輪一次給足五維與互動、技術需求；第二輪補響應式、心臟畫大、距離小、岩漿；第三輪心臟位置、跳動、點擊加速、鮮紅粒子、齒輪變慢；第四輪心臟 Y 軸置中；第五輪主動問「怎麼安排 graphic」後依序要求裂痕、火環、鐵籠；遇 script error 明確說「重來」並獲乾淨版本；最後一輪微調齒輪轉速對比。迭代有節奏、需求具體。</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>「響應式設計」「心臟畫大一點」「齒輪之間距離很小，幾乎有摩擦的感覺」「橘紅色的岩漿」；「心臟放在四個齒輪的正中間」「心臟變大又變小」「mouse left button click時…心臟…頻率暫時加速」「齒輪…變慢」；「重來，你遇到script error了」；「在還沒有按下mouse 之前，讓齒輪轉得比現在快一點」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>環境預見與判斷</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>需求含響應式、左鍵互動、多裝置／觸控；實作具 resize、心臟跳動與點擊加速、齒輪減速、岩漿／血液粒子、放射狀裂痕、火環、鐵籠、轉速對比，視覺層次與互動完整；技術面為逐步追加而非一次預見，故略扣一星。</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>「可以在任何的device打開都不失format」；AI 實作響應式、觸控、心臟跳動邏輯、齒輪減速、裂痕／火環／鐵籠繪製、轉速參數調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>生字內化與演化</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>能運用「質感」「明暗」「空間」「狹隘」「毛氈」「岩漿」「響應式」「心臟跳動」「齒輪摩擦」等語彙，並接受「壓抑的爆發」「摩擦壓迫感」等描述；主動引用 AI 提供的 brainstorm（lava, burning, cage）要求依序實作，生字內化與視覺演化清楚。</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>「質感是粗糙,像黑板的材質,毛氈」「空間是狹隘」「岩漿」；「缺少了一些你上面brain storm的idea, 比如說lava, burning file, cage」→ 先做1、接著做2、做3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>評分項目</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>使用 AI</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>得分 (4.2★)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>犀利點評</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>原文擷取 (學生指令)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>意圖解析與拆解</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>將「恐懼」具象化為呼吸式縮放、裂痕、長按層級、暗角與有機輪廓，規範完整且具互動藝術與氛圍感；需求條列清晰，技術方案（Canvas、CSS Variables、狀態管理）對應明確。</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>「我想要作互動式網頁，要符合以下規範：他是自適應網頁…滑鼠移動 &gt; 背景產生局部扭曲…長按 10 秒 &gt; 輪廓透明 25%…滾動 100% &gt; 畫面出現中央選擇區塊」</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>審美轉譯與內涵</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>以「氛圍感」「Atmospheric Horror」定位視覺風格，要求無裂痕/無輪廓的初始態與漸進揭露；後續接受程序化生成取代圖片，具象化有機輪廓與扭曲效果。</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>溝通效率與迭代</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>一次給足完整規範，AI 回覆即提供結構化方案與程式碼；追加「不用圖片、程式碼運算」與「完整 HTML」時能快速收斂為單一檔案實作。</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」「給我HTML完整程式碼」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>環境預見與判斷</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>需求已含自適應、多種輸入（滑鼠移動/點擊/長按/滾輪）與狀態累積（裂痕永久、輪廓殘留）；AI 建議震動動畫、效能最佳化與遮罩圖使用，具產品思維。</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>規範中已明確「自適應網頁」「滑鼠左鍵點擊（單擊）」「長按 1 秒 &gt; 畫面微震動」等層級與恢復條件</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>生字內化與演化</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>能運用「程序化生成」「Backdrop-filter」「Simplex Noise」等術語與 AI 回覆中的技術建議；需求從圖片改為純程式運算時表述清楚。</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>「不要用圖片改用程式碼運算」；對話中接受「Vanilla JS 搭配 CSS Variables」「requestAnimationFrame」等用語</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>評分項目</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>使用 AI</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>得分 (5.0★)</t>
         </is>
       </c>

</xml_diff>